<commit_message>
Fix database seeding order to resolve PostgreSQL foreign key violation on login
</commit_message>
<xml_diff>
--- a/backend/media/templates/loan_eligibility.xlsx
+++ b/backend/media/templates/loan_eligibility.xlsx
@@ -7,7 +7,8 @@
     <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" tabRatio="600" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
   </bookViews>
   <sheets>
-    <sheet name="Applications" sheetId="1" state="visible" r:id="rId1"/>
+    <sheet name="APRList" sheetId="1" state="visible" r:id="rId1"/>
+    <sheet name="Applications" sheetId="2" state="visible" r:id="rId2"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -135,21 +136,21 @@
       <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="4" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="right" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="4" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="4" fillId="4" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="4" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="right" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="4" fillId="5" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="left" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="5" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="4" fillId="4" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="right" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="4" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="left" vertical="center"/>
-    </xf>
     <xf numFmtId="0" fontId="5" fillId="0" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="5" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="6" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
@@ -519,6 +520,91 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
+  <dimension ref="A1:H7"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="15" customWidth="1" min="1" max="1"/>
+    <col width="20" customWidth="1" min="2" max="2"/>
+    <col width="12" customWidth="1" min="3" max="3"/>
+    <col width="12" customWidth="1" min="4" max="4"/>
+    <col width="12" customWidth="1" min="5" max="5"/>
+    <col width="12" customWidth="1" min="6" max="6"/>
+    <col width="12" customWidth="1" min="7" max="7"/>
+    <col width="12" customWidth="1" min="8" max="8"/>
+  </cols>
+  <sheetData>
+    <row r="1" ht="40" customHeight="1">
+      <c r="A1" s="1" t="inlineStr">
+        <is>
+          <t>INTERNAL FINANCE TRAINING: CREDIT TIER APR MATRIX</t>
+        </is>
+      </c>
+    </row>
+    <row r="2" ht="20" customHeight="1">
+      <c r="A2" s="2" t="inlineStr">
+        <is>
+          <t>Instructions: Fill in the empty highlighted cells using the requested Excel functions. Do NOT hardcode values.</t>
+        </is>
+      </c>
+    </row>
+    <row r="3" ht="15" customHeight="1"/>
+    <row r="4" ht="28" customHeight="1">
+      <c r="A4" s="3" t="inlineStr">
+        <is>
+          <t>Credit Tier</t>
+        </is>
+      </c>
+      <c r="B4" s="3" t="inlineStr">
+        <is>
+          <t>Standard APR (%)</t>
+        </is>
+      </c>
+    </row>
+    <row r="5" ht="22" customHeight="1">
+      <c r="A5" s="4" t="inlineStr">
+        <is>
+          <t>Excellent</t>
+        </is>
+      </c>
+      <c r="B5" s="5" t="n">
+        <v>0.0299</v>
+      </c>
+    </row>
+    <row r="6" ht="22" customHeight="1">
+      <c r="A6" s="6" t="inlineStr">
+        <is>
+          <t>Good</t>
+        </is>
+      </c>
+      <c r="B6" s="7" t="n">
+        <v>0.045</v>
+      </c>
+    </row>
+    <row r="7" ht="22" customHeight="1">
+      <c r="A7" s="4" t="inlineStr">
+        <is>
+          <t>Fair</t>
+        </is>
+      </c>
+      <c r="B7" s="5" t="n">
+        <v>0.0699</v>
+      </c>
+    </row>
+  </sheetData>
+  <mergeCells count="2">
+    <mergeCell ref="A2:H2"/>
+    <mergeCell ref="A1:H1"/>
+  </mergeCells>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
   <dimension ref="A1:I11"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
@@ -581,49 +667,49 @@
       </c>
     </row>
     <row r="5" ht="22" customHeight="1">
-      <c r="A5" s="4" t="n">
+      <c r="A5" s="5" t="n">
         <v>501</v>
       </c>
-      <c r="B5" s="5" t="inlineStr">
+      <c r="B5" s="4" t="inlineStr">
         <is>
           <t>Fatima</t>
         </is>
       </c>
-      <c r="C5" s="4" t="n">
+      <c r="C5" s="5" t="n">
         <v>12000</v>
       </c>
-      <c r="D5" s="5" t="inlineStr">
+      <c r="D5" s="4" t="inlineStr">
         <is>
           <t>Excellent</t>
         </is>
       </c>
-      <c r="E5" s="6" t="inlineStr"/>
-      <c r="F5" s="6" t="inlineStr"/>
-      <c r="H5" s="7" t="inlineStr">
+      <c r="E5" s="8" t="inlineStr"/>
+      <c r="F5" s="8" t="inlineStr"/>
+      <c r="H5" s="9" t="inlineStr">
         <is>
           <t>Audited Metrics:</t>
         </is>
       </c>
     </row>
     <row r="6" ht="22" customHeight="1">
-      <c r="A6" s="8" t="n">
+      <c r="A6" s="7" t="n">
         <v>502</v>
       </c>
-      <c r="B6" s="9" t="inlineStr">
+      <c r="B6" s="6" t="inlineStr">
         <is>
           <t>Sameer</t>
         </is>
       </c>
-      <c r="C6" s="8" t="n">
+      <c r="C6" s="7" t="n">
         <v>4500</v>
       </c>
-      <c r="D6" s="9" t="inlineStr">
+      <c r="D6" s="6" t="inlineStr">
         <is>
           <t>Good</t>
         </is>
       </c>
-      <c r="E6" s="6" t="inlineStr"/>
-      <c r="F6" s="6" t="inlineStr"/>
+      <c r="E6" s="8" t="inlineStr"/>
+      <c r="F6" s="8" t="inlineStr"/>
       <c r="H6" s="10" t="inlineStr">
         <is>
           <t>Approved Fair Credit Customers:</t>
@@ -632,44 +718,44 @@
       <c r="I6" s="11" t="n"/>
     </row>
     <row r="7" ht="22" customHeight="1">
-      <c r="A7" s="4" t="n">
+      <c r="A7" s="5" t="n">
         <v>503</v>
       </c>
-      <c r="B7" s="5" t="inlineStr">
+      <c r="B7" s="4" t="inlineStr">
         <is>
           <t>Jackson</t>
         </is>
       </c>
-      <c r="C7" s="4" t="n">
+      <c r="C7" s="5" t="n">
         <v>8000</v>
       </c>
-      <c r="D7" s="5" t="inlineStr">
+      <c r="D7" s="4" t="inlineStr">
         <is>
           <t>Fair</t>
         </is>
       </c>
-      <c r="E7" s="6" t="inlineStr"/>
-      <c r="F7" s="6" t="inlineStr"/>
+      <c r="E7" s="8" t="inlineStr"/>
+      <c r="F7" s="8" t="inlineStr"/>
     </row>
     <row r="8" ht="22" customHeight="1">
-      <c r="A8" s="8" t="n">
+      <c r="A8" s="7" t="n">
         <v>504</v>
       </c>
-      <c r="B8" s="9" t="inlineStr">
+      <c r="B8" s="6" t="inlineStr">
         <is>
           <t>Khadija</t>
         </is>
       </c>
-      <c r="C8" s="8" t="n">
+      <c r="C8" s="7" t="n">
         <v>15000</v>
       </c>
-      <c r="D8" s="9" t="inlineStr">
+      <c r="D8" s="6" t="inlineStr">
         <is>
           <t>Excellent</t>
         </is>
       </c>
-      <c r="E8" s="6" t="inlineStr"/>
-      <c r="F8" s="6" t="inlineStr"/>
+      <c r="E8" s="8" t="inlineStr"/>
+      <c r="F8" s="8" t="inlineStr"/>
       <c r="H8" s="12" t="inlineStr">
         <is>
           <t>Required formulas:</t>
@@ -677,24 +763,24 @@
       </c>
     </row>
     <row r="9" ht="22" customHeight="1">
-      <c r="A9" s="4" t="n">
+      <c r="A9" s="5" t="n">
         <v>505</v>
       </c>
-      <c r="B9" s="5" t="inlineStr">
+      <c r="B9" s="4" t="inlineStr">
         <is>
           <t>George</t>
         </is>
       </c>
-      <c r="C9" s="4" t="n">
+      <c r="C9" s="5" t="n">
         <v>5000</v>
       </c>
-      <c r="D9" s="5" t="inlineStr">
+      <c r="D9" s="4" t="inlineStr">
         <is>
           <t>Fair</t>
         </is>
       </c>
-      <c r="E9" s="6" t="inlineStr"/>
-      <c r="F9" s="6" t="inlineStr"/>
+      <c r="E9" s="8" t="inlineStr"/>
+      <c r="F9" s="8" t="inlineStr"/>
       <c r="H9" s="13" t="inlineStr">
         <is>
           <t>E5-E9: Status: 'Eligible' if Income &gt; 6000 and Tier != 'Fair' (IF, AND)</t>

</xml_diff>